<commit_message>
Execute Checkout test cases and refine wording
</commit_message>
<xml_diff>
--- a/Test-Cases/Test-Cases-Checkout.xlsx
+++ b/Test-Cases/Test-Cases-Checkout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0. Documentos\Github\qa-saucedemo-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35978DED-1D7B-44D4-AAA6-77345678557B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0770E4A7-D338-4EDE-9455-D29D3362584A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="82">
   <si>
     <t>ID</t>
   </si>
@@ -63,20 +63,10 @@
     <t>High</t>
   </si>
   <si>
-    <t>Given the user is logged in with products in the cart
-And the user is on the "Checkout: Your Information" form
-When they enter "Maria" in First Name, "Pimentel" in Last Name and "1097" in Zip/Postal Code
-And they click "Continue"
-Then the system should display the "Checkout: Overview" page showing the selected products</t>
-  </si>
-  <si>
     <t>Pass</t>
   </si>
   <si>
     <t>TC-002</t>
-  </si>
-  <si>
-    <t>First Name left empty is rejected</t>
   </si>
   <si>
     <t>Negative</t>
@@ -96,9 +86,6 @@
     <t>TC-003</t>
   </si>
   <si>
-    <t>Last Name left empty is rejected</t>
-  </si>
-  <si>
     <t>Given the user is logged in with products in the cart
 And the user is on the "Checkout: Your Information" form
 When they leave Last Name empty
@@ -110,9 +97,6 @@
     <t>TC-004</t>
   </si>
   <si>
-    <t>Zip/Postal Code left empty is rejected</t>
-  </si>
-  <si>
     <t>Given the user is logged in with products in the cart
 And the user is on the "Checkout: Your Information" form
 When they leave Zip/Postal Code empty
@@ -130,21 +114,7 @@
     <t>Low</t>
   </si>
   <si>
-    <t>Given the user is logged in with products in the cart
-And the user is on the "Checkout: Your Information" form
-When they leave two or more fields empty (all three fields; First Name and Last Name; First Name and Zip/Postal Code; Last Name and Zip/Postal Code)
-And they click "Continue"
-Then the system should block the action and display an error identifying a missing required field</t>
-  </si>
-  <si>
     <t>TC-006</t>
-  </si>
-  <si>
-    <t>Given the user is logged in with products in the cart
-And the user is on the "Checkout: Your Information" form
-When they enter "Maria" in First Name, "873729//*+" in Last Name and "1097" in Zip/Postal Code
-And they click "Continue"
-Then the system should reject the Last Name or display a message indicating that it contains invalid characters</t>
   </si>
   <si>
     <t>The system accepts the value and proceeds to the Overview with no warning.</t>
@@ -176,36 +146,16 @@
     <t>TC-009</t>
   </si>
   <si>
-    <t>Cancel from the information form returns to the cart keeping the products</t>
-  </si>
-  <si>
     <t>Edge case</t>
   </si>
   <si>
-    <t>Given the user is logged in with products in the cart
-And the user is on the "Checkout: Your Information" form
-When they click the "Cancel" button
-Then the system should return the user to the cart with the products still listed</t>
-  </si>
-  <si>
     <t>TC-010</t>
   </si>
   <si>
-    <t>Cancel from the Overview keeps the products in the cart</t>
-  </si>
-  <si>
-    <t>Given the user is on the "Checkout: Overview" page with 2 products
-When they click the "Cancel" button
-Then the system should abandon the checkout and keep both products in the cart</t>
-  </si>
-  <si>
     <t>TC-011</t>
   </si>
   <si>
     <t>TC-012</t>
-  </si>
-  <si>
-    <t>Direct access to the Overview without an active session</t>
   </si>
   <si>
     <t>Negative / Security</t>
@@ -219,17 +169,7 @@
     <t>TC-013</t>
   </si>
   <si>
-    <t>Given the user is logged in, has products in the cart and is on the inventory page
-When they manually enter the URL "https://www.saucedemo.com/checkout-step-two.html"
-Then the system should not allow skipping the information form, and should redirect the user to it or block the access</t>
-  </si>
-  <si>
     <t>TC-014</t>
-  </si>
-  <si>
-    <t>Given the user is logged in, has no products in the cart and is on the inventory page
-When they manually enter the URL "https://www.saucedemo.com/checkout-step-two.html"
-Then the system should not allow reaching the Overview or finishing an order with no products</t>
   </si>
   <si>
     <t>The Overview page is displayed with the selected products.</t>
@@ -263,54 +203,140 @@
     <t>Item total, tax and total are consistent ($39.98 + $3.20 = $43.18).</t>
   </si>
   <si>
-    <t>The user returns to the cart with the products preserved.</t>
-  </si>
-  <si>
-    <t>The user returns to the inventory with the same 2 products still in the cart.</t>
-  </si>
-  <si>
     <t>Finish the order from the Overview</t>
   </si>
   <si>
-    <t>Given the user is on the "Checkout: Overview" page with products in the cart
+    <t>The message "Thank you for your order!" is displayed.</t>
+  </si>
+  <si>
+    <t>Return to the inventory after completing an order</t>
+  </si>
+  <si>
+    <t>The inventory is displayed with the cart at 0.</t>
+  </si>
+  <si>
+    <t>TC-015</t>
+  </si>
+  <si>
+    <t>The access is blocked with the message "Epic sadface: You can only access '/checkout-step-two.html' when you are logged in."</t>
+  </si>
+  <si>
+    <t>The action is blocked, but only one error is shown: the one for the first empty field (e.g. "Error: First Name is required" when all three are empty).</t>
+  </si>
+  <si>
+    <t>Leave the information form and return to the cart</t>
+  </si>
+  <si>
+    <t>The user returns to the cart with the products preserved when leaving with the "Cancel" button and with the browser's back arrow.</t>
+  </si>
+  <si>
+    <t>Cancel the checkout from the Overview page</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with "Sauce Labs Backpack" and "Sauce Labs Bike Light" in the cart
+And the user is on the "Checkout: Overview" page
+When they click the "Cancel" button
+Then the system should return the user to the inventory page
+And both products should remain in the cart</t>
+  </si>
+  <si>
+    <t>The user returns to the inventory page and both products remain in the cart.</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with "Sauce Labs Backpack" and "Sauce Labs Bike Light" in the cart
+And the user is on the "Checkout: Overview" page
 When they click the "Finish" button
 Then the system should display a confirmation message indicating that the order was placed</t>
   </si>
   <si>
-    <t>The message "Thank you for your order!" is displayed.</t>
-  </si>
-  <si>
-    <t>Return to the inventory after completing an order</t>
-  </si>
-  <si>
-    <t>Given the user has completed an order and is on the order confirmation page
+    <t>The Overview page opens even though the information form was not completed.</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with no products in the cart
+And the user is on the inventory page
+When they manually enter the URL "https://www.saucedemo.com/checkout-step-two.html" in the browser
+Then the system should not allow reaching the Overview page without products in the cart</t>
+  </si>
+  <si>
+    <t>The Overview page opens with no products.</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with "Sauce Labs Backpack" and "Sauce Labs Bike Light" in the cart
+And the user is on the inventory page
+And the user has not completed the "Checkout: Your Information" form
+When they manually enter the URL "https://www.saucedemo.com/checkout-step-two.html" in the browser
+Then the system should not display the Overview page
+And the system should redirect the user to the information form</t>
+  </si>
+  <si>
+    <t>TC-016</t>
+  </si>
+  <si>
+    <t>Given the user is logged in and has completed an order with "Sauce Labs Backpack" and "Sauce Labs Bike Light"
+And the user entered "Maria", "Pimentel" and "1097" as first name, last name and zip/postal code in the information form
+And the user is on the "Checkout: Complete!" page
+When they click the "Generate PDF order" button
+Then the system should generate a PDF order
+And the PDF should list both products with their prices ($29.99 and $9.99)
+And the PDF should show the same item total, tax and total as the Overview ($39.98, $3.20 and $43.18)
+And the PDF should show the first name, last name and zip/postal code entered in the form</t>
+  </si>
+  <si>
+    <t>The PDF lists both products with their prices, the item total, the tax, the total and the first name, last name and zip code entered in the form.</t>
+  </si>
+  <si>
+    <t>Generate the PDF order from the confirmation page</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with products in the cart
+And the user is on the "Checkout: Your Information" form
+When they enter "Maria" in First Name, "873729//*+" in Last Name and "1097" in Zip/Postal Code
+And they click "Continue"
+Then the system should not accept the Last Name and should display a message indicating that it contains invalid characters</t>
+  </si>
+  <si>
+    <t>First Name left empty</t>
+  </si>
+  <si>
+    <t>Last Name left empty</t>
+  </si>
+  <si>
+    <t>Direct access to the Overview page by URL without completing the information form</t>
+  </si>
+  <si>
+    <t>Direct access to the Overview page by URL with an empty cart</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with "Sauce Labs Backpack" and "Sauce Labs Bike Light" in the cart
+And the user is on the "Checkout: Your Information" form
+When they enter "Maria" in First Name, "Pimentel" in Last Name and "1097" in Zip/Postal Code
+And they click "Continue"
+Then the system should display the "Checkout: Overview" page showing the selected products</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with "Sauce Labs Backpack" and "Sauce Labs Bike Light" in the cart
+And the user is on the "Checkout: Your Information" form
+When they leave the form using each of these options, one at a time: the "Cancel" button and the browser's back arrow
+Then in both cases the system should return the user to the cart with the products still listed</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with products in the cart
+And the user is on the "Checkout: Your Information" form
+When they leave empty each of these field combinations, one at a time: all three fields; First Name and Last Name; First Name and Zip/Postal Code; Last Name and Zip/Postal Code
+And they click "Continue"
+Then in all cases the system should block the action and display an error identifying a missing required field</t>
+  </si>
+  <si>
+    <t>Given the user has completed an order and is on the "Checkout: Complete!" page
 When they click the "Back Home" button
-Then the system should return the user to the inventory
+Then the system should return the user to the inventory page
 And the cart should be empty</t>
   </si>
   <si>
-    <t>The inventory is displayed with the cart at 0.</t>
-  </si>
-  <si>
-    <t>TC-015</t>
-  </si>
-  <si>
-    <t>Direct access to the Overview skipping the information form (with products in cart)</t>
-  </si>
-  <si>
-    <t>The system opens the Overview without the form being completed and allows the purchase to be finished.</t>
-  </si>
-  <si>
-    <t>Direct access to the Overview with an empty cart</t>
-  </si>
-  <si>
-    <t>The system opens the Overview with no products and without the form being completed, and allows the purchase to be finished.</t>
-  </si>
-  <si>
-    <t>The access is blocked with the message "Epic sadface: You can only access '/checkout-step-two.html' when you are logged in."</t>
-  </si>
-  <si>
-    <t>The action is blocked, but only one error is shown: the one for the first empty field (e.g. "Error: First Name is required" when all three are empty).</t>
+    <t>Zip/Postal Code left empty</t>
+  </si>
+  <si>
+    <t>Direct access to the Overview page by URL without an active session</t>
   </si>
 </sst>
 </file>
@@ -318,7 +344,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -437,13 +463,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -747,7 +773,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="108.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -761,180 +787,180 @@
         <v>11</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="F3" s="3" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H3" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H5" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>27</v>
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="H7" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="H8" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>10</v>
@@ -943,76 +969,76 @@
         <v>11</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="10">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="10">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="88.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="10">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="10">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>64</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H11" s="10">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>10</v>
@@ -1021,126 +1047,152 @@
         <v>11</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H12" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H13" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H14" s="10">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="H15" s="10">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="87" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="H16" s="10">
-        <v>46303</v>
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="169.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="10">
+        <v>46308</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G16" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G17" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail,Blocked,Pending"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>